<commit_message>
feat(customers): support importing customer ledgers from external accounting apps with opening balances
</commit_message>
<xml_diff>
--- a/tools/external_customers_sample.xlsx
+++ b/tools/external_customers_sample.xlsx
@@ -2,36 +2,39 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="العملاء والمشتركون" sheetId="1" r:id="rId1"/>
+    <sheet name="كشف حسابات العملاء" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="230">
   <si>
     <t>م</t>
   </si>
   <si>
-    <t>اسم العميل</t>
+    <t>اسم الحساب</t>
   </si>
   <si>
     <t>رقم الهاتف</t>
   </si>
   <si>
-    <t>اسم المزرعة</t>
-  </si>
-  <si>
-    <t>الموقع</t>
-  </si>
-  <si>
-    <t>سعر الساعة</t>
-  </si>
-  <si>
-    <t>نوع الحساب</t>
-  </si>
-  <si>
-    <t>ملاحظات</t>
+    <t>العنوان</t>
+  </si>
+  <si>
+    <t>الرصيد الحالي</t>
+  </si>
+  <si>
+    <t>الحالة</t>
+  </si>
+  <si>
+    <t>العملة</t>
+  </si>
+  <si>
+    <t>تاريخ آخر حركة</t>
+  </si>
+  <si>
+    <t>ملاحظات / البيان</t>
   </si>
   <si>
     <t>صالح أحمد بن علي العولقي</t>
@@ -40,16 +43,19 @@
     <t>771234001</t>
   </si>
   <si>
-    <t>مزرعة وادي سهام</t>
-  </si>
-  <si>
     <t>الحديدة - باجل</t>
   </si>
   <si>
-    <t>عميل عادي</t>
-  </si>
-  <si>
-    <t>مشترك رئيسي - زراعة طماطم وبصل</t>
+    <t>مطلوب منه (مدين)</t>
+  </si>
+  <si>
+    <t>ريال يمني</t>
+  </si>
+  <si>
+    <t>2026/09/25</t>
+  </si>
+  <si>
+    <t>باقي حساب سقي طماطم وبصل لشهر 9</t>
   </si>
   <si>
     <t>عبد الله محمد بن ناصر الحميري</t>
@@ -58,13 +64,13 @@
     <t>772345002</t>
   </si>
   <si>
-    <t>حقل الجربة الكبرى</t>
-  </si>
-  <si>
     <t>ذمار - رداع</t>
   </si>
   <si>
-    <t>ري بالتقطير - حقل ذرة</t>
+    <t>2026/10/01</t>
+  </si>
+  <si>
+    <t>أجور ري حقل الذرة - الموسم الخريفي</t>
   </si>
   <si>
     <t>محمد يحيى بن سالم السالمي</t>
@@ -73,16 +79,16 @@
     <t>773456003</t>
   </si>
   <si>
-    <t>بستان العنب والنخيل</t>
-  </si>
-  <si>
     <t>صنعاء - بني حشيش</t>
   </si>
   <si>
-    <t>صاحب بئر</t>
-  </si>
-  <si>
-    <t>مالك بئر الوادي المشترك</t>
+    <t>مطلوب له (دائن)</t>
+  </si>
+  <si>
+    <t>2026/10/03</t>
+  </si>
+  <si>
+    <t>دفعة مقدمة تحت الحساب لبستان العنب</t>
   </si>
   <si>
     <t>علي حسين بن قاسم الريمي</t>
@@ -91,13 +97,13 @@
     <t>774567004</t>
   </si>
   <si>
-    <t>مزرعة الجرادين</t>
-  </si>
-  <si>
     <t>إب - السحول</t>
   </si>
   <si>
-    <t>محاصيل حبوب وخضار</t>
+    <t>2026/09/18</t>
+  </si>
+  <si>
+    <t>حساب سقي حبوب وخضار قاع الحقل</t>
   </si>
   <si>
     <t>أحمد سالم بن عبده الزبيدي</t>
@@ -106,10 +112,10 @@
     <t>775678005</t>
   </si>
   <si>
-    <t>مزرعة باجل الشرقية</t>
-  </si>
-  <si>
-    <t>سقي منتظم كل أسبوعين</t>
+    <t>2026/10/04</t>
+  </si>
+  <si>
+    <t>سقي منتظم كل أسبوعين - دفعة مؤجلة</t>
   </si>
   <si>
     <t>يحيى إبراهيم بن مسعد الكندي</t>
@@ -118,13 +124,13 @@
     <t>776789006</t>
   </si>
   <si>
-    <t>حقل العرج والساحل</t>
-  </si>
-  <si>
     <t>الحديدة - بيت الفقيه</t>
   </si>
   <si>
-    <t>أشجار نخيل ومانجو</t>
+    <t>2026/09/20</t>
+  </si>
+  <si>
+    <t>ري نخيل وأشجار مانجو موسم الصيف</t>
   </si>
   <si>
     <t>حسين عمر بن سعيد اليافعي</t>
@@ -133,13 +139,13 @@
     <t>777890007</t>
   </si>
   <si>
-    <t>مزرعة وادي مور</t>
-  </si>
-  <si>
     <t>حجة - عبس</t>
   </si>
   <si>
-    <t>مضخة فرعية للشبكة</t>
+    <t>2026/09/28</t>
+  </si>
+  <si>
+    <t>أجور ساعات ماء للشبكة الفرعية</t>
   </si>
   <si>
     <t>إبراهيم منصور بن حسين الحبيشي</t>
@@ -148,13 +154,13 @@
     <t>778901008</t>
   </si>
   <si>
-    <t>بستان الضالع</t>
-  </si>
-  <si>
     <t>لحج - تبن</t>
   </si>
   <si>
-    <t>شريك في تشغيل البئر الغربي</t>
+    <t>2026/10/02</t>
+  </si>
+  <si>
+    <t>مستحقات تشغيل وتغذية بئر غربي</t>
   </si>
   <si>
     <t>سالم خالد بن منصور الشميري</t>
@@ -163,13 +169,13 @@
     <t>779012009</t>
   </si>
   <si>
-    <t>مزرعة العواذل</t>
-  </si>
-  <si>
     <t>أبين - دلتا</t>
   </si>
   <si>
-    <t>زراعة أعلاف وموز</t>
+    <t>2026/09/15</t>
+  </si>
+  <si>
+    <t>ري مزارع أعلاف وموز دلتا أبين</t>
   </si>
   <si>
     <t>عمر عادل بن علي التهامي</t>
@@ -178,13 +184,13 @@
     <t>770123010</t>
   </si>
   <si>
-    <t>حقل الخضراء</t>
-  </si>
-  <si>
     <t>الحديدة - المراوعة</t>
   </si>
   <si>
-    <t>ري صباحي دوري</t>
+    <t>2026/10/05</t>
+  </si>
+  <si>
+    <t>ري صباحي دوري - متبقي الدفعة الأولى</t>
   </si>
   <si>
     <t>منصور طارق بن ناصر الأهدل</t>
@@ -193,13 +199,13 @@
     <t>733456011</t>
   </si>
   <si>
-    <t>مزرعة الساحل الغربي</t>
-  </si>
-  <si>
     <t>الحديدة - الدريهمي</t>
   </si>
   <si>
-    <t>حقل خضروات مشكلة</t>
+    <t>2026/09/22</t>
+  </si>
+  <si>
+    <t>سقي خضروات مشكلة وحقل بطاطا</t>
   </si>
   <si>
     <t>خالد فؤاد بن أحمد الصبيحي</t>
@@ -208,13 +214,13 @@
     <t>734567012</t>
   </si>
   <si>
-    <t>بستان الخير والبركة</t>
-  </si>
-  <si>
     <t>لحج - طور الباحة</t>
   </si>
   <si>
-    <t>زراعة حبوب صيفية</t>
+    <t>2026/09/30</t>
+  </si>
+  <si>
+    <t>أجور ري حبوب صيفية</t>
   </si>
   <si>
     <t>عادل رمزي بن سالم البركاني</t>
@@ -223,13 +229,13 @@
     <t>735678013</t>
   </si>
   <si>
-    <t>مزرعة الروضة</t>
-  </si>
-  <si>
     <t>تعز - الشمايتين</t>
   </si>
   <si>
-    <t>بئر البركاني المغذي لخط 2</t>
+    <t>2026/10/06</t>
+  </si>
+  <si>
+    <t>مستحقات شراء ماء شبكة من بئر البركاني</t>
   </si>
   <si>
     <t>ياسر وليد بن حسن المخلافي</t>
@@ -238,13 +244,13 @@
     <t>736789014</t>
   </si>
   <si>
-    <t>حقل وادي بنا</t>
-  </si>
-  <si>
     <t>إب - النادرة</t>
   </si>
   <si>
-    <t>مزارع ذرة وبقوليات</t>
+    <t>2026/09/19</t>
+  </si>
+  <si>
+    <t>ري حقول ذرة وبقوليات وادي بنا</t>
   </si>
   <si>
     <t>طارق فيصل بن قاسم الشوافي</t>
@@ -253,13 +259,10 @@
     <t>737890015</t>
   </si>
   <si>
-    <t>مزرعة سهول تهامة</t>
-  </si>
-  <si>
     <t>الحديدة - الزيدية</t>
   </si>
   <si>
-    <t>مشترك جديد موسم أول</t>
+    <t>حساب ري سهول تهامة الموسم الأول</t>
   </si>
   <si>
     <t>فؤاد مجيب بن عبده الضبياني</t>
@@ -268,13 +271,13 @@
     <t>738901016</t>
   </si>
   <si>
-    <t>بستان الموز والمانجو</t>
-  </si>
-  <si>
     <t>أبين - جعار</t>
   </si>
   <si>
-    <t>بستان مانجو مثمر</t>
+    <t>2026/09/27</t>
+  </si>
+  <si>
+    <t>ري بستان مانجو مثمر</t>
   </si>
   <si>
     <t>رمزي عصام بن مسعد الردفاني</t>
@@ -283,13 +286,10 @@
     <t>739012017</t>
   </si>
   <si>
-    <t>مزرعة الردفان الخضراء</t>
-  </si>
-  <si>
     <t>لحج - ردفان</t>
   </si>
   <si>
-    <t>سقي ليلي بنصف القيمة</t>
+    <t>سقي ليلي مخفض لحقل الأعلاف</t>
   </si>
   <si>
     <t>وليد هائل بن سعيد الأنسي</t>
@@ -298,13 +298,13 @@
     <t>730123018</t>
   </si>
   <si>
-    <t>حقل قاع جهران</t>
-  </si>
-  <si>
     <t>ذمار - جهران</t>
   </si>
   <si>
-    <t>مالك بئر السلام الرئيسي</t>
+    <t>2026/10/07</t>
+  </si>
+  <si>
+    <t>حساب توريد وتغذية مياه قاع جهران</t>
   </si>
   <si>
     <t>فيصل عبد الرقيب بن حسين القحوم</t>
@@ -313,13 +313,13 @@
     <t>711234019</t>
   </si>
   <si>
-    <t>مزرعة شبوة الشرقية</t>
-  </si>
-  <si>
     <t>مأرب - الوادي</t>
   </si>
   <si>
-    <t>زراعة قمح وبر</t>
+    <t>2026/09/24</t>
+  </si>
+  <si>
+    <t>ري محصول القمح والبر الصحراوي</t>
   </si>
   <si>
     <t>مجيب قائد بن منصور السيد</t>
@@ -328,10 +328,7 @@
     <t>712345020</t>
   </si>
   <si>
-    <t>بستان الحسينية</t>
-  </si>
-  <si>
-    <t>بستان حمضيات ونخيل</t>
+    <t>سقي بستان حمضيات ونخيل الحسينية</t>
   </si>
   <si>
     <t>عصام مقبل بن علي الهدار</t>
@@ -340,13 +337,13 @@
     <t>713456021</t>
   </si>
   <si>
-    <t>مزرعة الوادي الكبير</t>
-  </si>
-  <si>
     <t>حضرموت - تريم</t>
   </si>
   <si>
-    <t>نظام ري محوري</t>
+    <t>2026/09/17</t>
+  </si>
+  <si>
+    <t>تشغيل ري محوري لمحاصيل الأعلاف</t>
   </si>
   <si>
     <t>هائل ناجي بن ناصر الشيباني</t>
@@ -355,13 +352,13 @@
     <t>714567022</t>
   </si>
   <si>
-    <t>حقل ذمار القرن</t>
-  </si>
-  <si>
     <t>ذمار - عنس</t>
   </si>
   <si>
-    <t>حقول بطاطس وبقوليات</t>
+    <t>2026/09/29</t>
+  </si>
+  <si>
+    <t>ري حقول بطاطس وبقوليات ذمار القرن</t>
   </si>
   <si>
     <t>عبد الرقيب زيد بن أحمد السنحاني</t>
@@ -370,13 +367,10 @@
     <t>715678023</t>
   </si>
   <si>
-    <t>بستان سنحان الجميل</t>
-  </si>
-  <si>
     <t>صنعاء - سنحان</t>
   </si>
   <si>
-    <t>تغذية خزانات القرية</t>
+    <t>مستحقات بئر مياه سنحان المغذي للقرية</t>
   </si>
   <si>
     <t>قائد عبده بن سالم الخولاني</t>
@@ -385,13 +379,13 @@
     <t>716789024</t>
   </si>
   <si>
-    <t>مزرعة جبال خولان</t>
-  </si>
-  <si>
     <t>صنعاء - خولان</t>
   </si>
   <si>
-    <t>مدرجات لوز وبن</t>
+    <t>2026/09/21</t>
+  </si>
+  <si>
+    <t>ري مدرجات اللوز والبن الجبلي</t>
   </si>
   <si>
     <t>مقبل سعيد بن حسن الهمداني</t>
@@ -400,13 +394,13 @@
     <t>717890025</t>
   </si>
   <si>
-    <t>حقل قاع المنقب</t>
-  </si>
-  <si>
     <t>صنعاء - همدان</t>
   </si>
   <si>
-    <t>حقول خضار موسمية</t>
+    <t>2026/09/26</t>
+  </si>
+  <si>
+    <t>أجور سقي خضار موسمية قاع المنقب</t>
   </si>
   <si>
     <t>ناجي صابر بن قاسم الوصابي</t>
@@ -415,13 +409,10 @@
     <t>718901026</t>
   </si>
   <si>
-    <t>مزرعة وصاب العالي</t>
-  </si>
-  <si>
     <t>ذمار - وصاب</t>
   </si>
   <si>
-    <t>سقي تكميلي للأشجار</t>
+    <t>ري تكميلي لأشجار البن والفواكه</t>
   </si>
   <si>
     <t>زيد جميل بن عبده الجعدي</t>
@@ -430,13 +421,13 @@
     <t>719012027</t>
   </si>
   <si>
-    <t>بستان دوعن الفسيح</t>
-  </si>
-  <si>
     <t>حضرموت - دوعن</t>
   </si>
   <si>
-    <t>نخيل ومناحل عسل</t>
+    <t>2026/09/16</t>
+  </si>
+  <si>
+    <t>سقي نخيل ومناحل سدر وادي دوعن</t>
   </si>
   <si>
     <t>عبده توفيق بن مسعد المشرقي</t>
@@ -445,13 +436,10 @@
     <t>710123028</t>
   </si>
   <si>
-    <t>حقل حيران الأخضر</t>
-  </si>
-  <si>
     <t>حجة - حيران</t>
   </si>
   <si>
-    <t>زراعة بصل وسمسم</t>
+    <t>ري حقول بصل وسمسم حيران</t>
   </si>
   <si>
     <t>سعيد صالح بن سعيد الحميلي</t>
@@ -460,10 +448,10 @@
     <t>771122029</t>
   </si>
   <si>
-    <t>مزرعة النور والبركة</t>
-  </si>
-  <si>
-    <t>بئر النور الارتوازي</t>
+    <t>2026/10/08</t>
+  </si>
+  <si>
+    <t>مستحقات توريد مياه ارتوازية من بئر النور</t>
   </si>
   <si>
     <t>صابر عبد الله بن علي الجبلي</t>
@@ -472,13 +460,13 @@
     <t>772233030</t>
   </si>
   <si>
-    <t>بستان وادي السحتين</t>
-  </si>
-  <si>
     <t>إب - جبلة</t>
   </si>
   <si>
-    <t>مدرجات بن وخضار</t>
+    <t>2026/09/23</t>
+  </si>
+  <si>
+    <t>ري مدرجات بن وخضار وادي السحتين</t>
   </si>
   <si>
     <t>جميل محمد بن ناصر الصالحي</t>
@@ -487,13 +475,10 @@
     <t>773344031</t>
   </si>
   <si>
-    <t>حقل الخيرات الوفيرة</t>
-  </si>
-  <si>
     <t>لحج - الحوطة</t>
   </si>
   <si>
-    <t>مزارع ذرة رفيعة</t>
+    <t>أجور سقي حقول ذرة رفيعة</t>
   </si>
   <si>
     <t>توفيق أحمد بن سالم النمري</t>
@@ -502,13 +487,13 @@
     <t>774455032</t>
   </si>
   <si>
-    <t>مزرعة الجوف الشمالية</t>
-  </si>
-  <si>
     <t>مأرب - الجوبة</t>
   </si>
   <si>
-    <t>قمح وشعير مسقى</t>
+    <t>2026/09/14</t>
+  </si>
+  <si>
+    <t>ري مزارع القمح والشعير</t>
   </si>
   <si>
     <t>صالح يحيى بن أحمد العنسي</t>
@@ -517,10 +502,7 @@
     <t>775566033</t>
   </si>
   <si>
-    <t>حقل عنس الأوسط</t>
-  </si>
-  <si>
-    <t>حقول بطاطس مسقية</t>
+    <t>ري حقول بطاطس عنس الأوسط</t>
   </si>
   <si>
     <t>عبد الله إبراهيم بن حسن البكاري</t>
@@ -529,13 +511,10 @@
     <t>776677034</t>
   </si>
   <si>
-    <t>مزرعة وادي سردد</t>
-  </si>
-  <si>
     <t>المحويت - شبام</t>
   </si>
   <si>
-    <t>بساتين بن وفواكه</t>
+    <t>سقي بساتين بن وفواكه وادي سردد</t>
   </si>
   <si>
     <t>محمد سالم بن قاسم الحرازي</t>
@@ -544,13 +523,10 @@
     <t>777788035</t>
   </si>
   <si>
-    <t>بستان مناخة الخضراء</t>
-  </si>
-  <si>
     <t>صنعاء - حراز</t>
   </si>
   <si>
-    <t>بئر مياه عذبة للشبكة</t>
+    <t>مستحقات توريد مياه عذبة للشبكة</t>
   </si>
   <si>
     <t>علي عمر بن عبده الحكيمي</t>
@@ -559,10 +535,7 @@
     <t>778899036</t>
   </si>
   <si>
-    <t>حقل التربة الأعلى</t>
-  </si>
-  <si>
-    <t>سقي منتظم بالصهاريج</t>
+    <t>أجور سقي بالصهاريج للتربة الأعلى</t>
   </si>
   <si>
     <t>أحمد منصور بن مسعد الدبعي</t>
@@ -571,13 +544,10 @@
     <t>779900037</t>
   </si>
   <si>
-    <t>مزرعة ذبحان النموذجية</t>
-  </si>
-  <si>
     <t>تعز - المعافر</t>
   </si>
   <si>
-    <t>حقل ذرة وأشجار مثمرة</t>
+    <t>حساب ري حقل ذرة وأشجار مثمرة</t>
   </si>
   <si>
     <t>يحيى خالد بن سعيد الشرجبي</t>
@@ -586,13 +556,10 @@
     <t>771020038</t>
   </si>
   <si>
-    <t>بستان شوافي الصعيد</t>
-  </si>
-  <si>
     <t>تعز - صبر الموادم</t>
   </si>
   <si>
-    <t>مدرجات خضار فواكه</t>
+    <t>سقي مدرجات فواكه وخضار الصعيد</t>
   </si>
   <si>
     <t>حسين عادل بن علي المقالح</t>
@@ -601,13 +568,10 @@
     <t>772030039</t>
   </si>
   <si>
-    <t>مزرعة قاع المقالح</t>
-  </si>
-  <si>
     <t>إب - يريم</t>
   </si>
   <si>
-    <t>محاصيل حبوب شتوية</t>
+    <t>ري محاصيل حبوب قاع المقالح الشتوية</t>
   </si>
   <si>
     <t>إبراهيم طارق بن ناصر الوادعي</t>
@@ -616,13 +580,10 @@
     <t>773040040</t>
   </si>
   <si>
-    <t>حقل دماج الخصيب</t>
-  </si>
-  <si>
     <t>صعدة - الصفراء</t>
   </si>
   <si>
-    <t>بستان رمان وعنب صعدي</t>
+    <t>ري بساتين رمان وعنب صعدي دماج</t>
   </si>
   <si>
     <t>سالم فؤاد بن أحمد الخضري</t>
@@ -631,13 +592,10 @@
     <t>774050041</t>
   </si>
   <si>
-    <t>مزرعة زبيد التاريخية</t>
-  </si>
-  <si>
     <t>الحديدة - زبيد</t>
   </si>
   <si>
-    <t>بئر زبيد الزراعي</t>
+    <t>مستحقات تشغيل بئر زبيد الزراعي</t>
   </si>
   <si>
     <t>عمر رمزي بن سالم المعمري</t>
@@ -646,10 +604,7 @@
     <t>775060042</t>
   </si>
   <si>
-    <t>حقل المعافر الأوسط</t>
-  </si>
-  <si>
-    <t>سقي خضار وسمسم</t>
+    <t>أجور ري سمسم وخضار المعافر الأوسط</t>
   </si>
   <si>
     <t>منصور وليد بن حسن الصامت</t>
@@ -658,13 +613,10 @@
     <t>776070043</t>
   </si>
   <si>
-    <t>بستان وادي المعاين</t>
-  </si>
-  <si>
     <t>إب - المشنة</t>
   </si>
   <si>
-    <t>خضروات ورقية وبطاطس</t>
+    <t>سقي خضروات ورقية وبطاطس وادي المعاين</t>
   </si>
   <si>
     <t>خالد فيصل بن قاسم اليافعي</t>
@@ -673,13 +625,10 @@
     <t>777080044</t>
   </si>
   <si>
-    <t>مزرعة ردفان الجنوبية</t>
-  </si>
-  <si>
     <t>لحج - حبيل جبر</t>
   </si>
   <si>
-    <t>مزارع ذرة وأعلاف مواشي</t>
+    <t>ري مزارع ذرة وأعلاف مواشي ردفان</t>
   </si>
   <si>
     <t>عادل مجيب بن عبده الحريبي</t>
@@ -688,13 +637,10 @@
     <t>778090045</t>
   </si>
   <si>
-    <t>حقل خبت الرجاع</t>
-  </si>
-  <si>
     <t>لحج - المضاربة</t>
   </si>
   <si>
-    <t>ري أحواض موسمية</t>
+    <t>أجور ري أحواض موسمية خبت الرجاع</t>
   </si>
   <si>
     <t>ياسر عصام بن مسعد المسوري</t>
@@ -703,13 +649,10 @@
     <t>779010046</t>
   </si>
   <si>
-    <t>مزرعة جبل مسور</t>
-  </si>
-  <si>
     <t>عمران - مسور</t>
   </si>
   <si>
-    <t>مالك بئر المحطة</t>
+    <t>مستحقات بئر مياه محطة جبل مسور</t>
   </si>
   <si>
     <t>طارق هائل بن سعيد الأهدل</t>
@@ -718,13 +661,10 @@
     <t>770120047</t>
   </si>
   <si>
-    <t>بستان المنصورية الرطب</t>
-  </si>
-  <si>
     <t>الحديدة - المنصورية</t>
   </si>
   <si>
-    <t>أشجار مانجو بلدي وموز</t>
+    <t>سقي أشجار مانجو بلدي وموز المنصورية</t>
   </si>
   <si>
     <t>فؤاد عبد الرقيب بن حسين الذماري</t>
@@ -733,13 +673,10 @@
     <t>731230048</t>
   </si>
   <si>
-    <t>حقل وادي زراجة</t>
-  </si>
-  <si>
     <t>ذمار - الحداء</t>
   </si>
   <si>
-    <t>زراعة ثوم وبصل وحبوب</t>
+    <t>ري محصول الثوم والبصل وادي زراجة</t>
   </si>
   <si>
     <t>رمزي قائد بن منصور الكبسي</t>
@@ -748,10 +685,7 @@
     <t>732340049</t>
   </si>
   <si>
-    <t>مزرعة قاع سهمان</t>
-  </si>
-  <si>
-    <t>بساتين مشمش ولوز</t>
+    <t>سقي بساتين مشمش ولوز قاع سهمان</t>
   </si>
   <si>
     <t>وليد مقبل بن علي الحيدري</t>
@@ -760,10 +694,10 @@
     <t>733450050</t>
   </si>
   <si>
-    <t>حقل ضوران الأشمور</t>
-  </si>
-  <si>
     <t>عمران - خارف</t>
+  </si>
+  <si>
+    <t>ري محاصيل حبوب وخضار ضوران الأشمور</t>
   </si>
 </sst>
 </file>
@@ -796,31 +730,37 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="F2">
-        <v>3000</v>
+      <c r="E2">
+        <v>45000</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -828,25 +768,28 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3">
-        <v>3500</v>
+        <v>18</v>
+      </c>
+      <c r="E3">
+        <v>28500</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -854,25 +797,28 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4">
-        <v>4000</v>
+        <v>23</v>
+      </c>
+      <c r="E4">
+        <v>15000</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="I4" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -880,25 +826,28 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5">
-        <v>3000</v>
+        <v>29</v>
+      </c>
+      <c r="E5">
+        <v>62000</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
       </c>
       <c r="G5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H5" t="s">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="I5" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="6">
@@ -906,25 +855,28 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" t="s">
         <v>11</v>
       </c>
-      <c r="F6">
-        <v>3200</v>
+      <c r="E6">
+        <v>18000</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
       </c>
       <c r="G6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H6" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="I6" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -932,25 +884,28 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7">
-        <v>2800</v>
+        <v>38</v>
+      </c>
+      <c r="E7">
+        <v>53000</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
       </c>
       <c r="G7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H7" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="I7" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -958,25 +913,28 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8">
-        <v>3500</v>
+        <v>43</v>
+      </c>
+      <c r="E8">
+        <v>34000</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
       </c>
       <c r="G8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H8" t="s">
-        <v>43</v>
+        <v>44</v>
+      </c>
+      <c r="I8" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="9">
@@ -984,25 +942,28 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E9" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9">
-        <v>3000</v>
+        <v>48</v>
+      </c>
+      <c r="E9">
+        <v>22000</v>
+      </c>
+      <c r="F9" t="s">
+        <v>24</v>
       </c>
       <c r="G9" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="H9" t="s">
-        <v>48</v>
+        <v>49</v>
+      </c>
+      <c r="I9" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="10">
@@ -1010,25 +971,28 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D10" t="s">
-        <v>51</v>
-      </c>
-      <c r="E10" t="s">
-        <v>52</v>
-      </c>
-      <c r="F10">
-        <v>3200</v>
+        <v>53</v>
+      </c>
+      <c r="E10">
+        <v>41500</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
       </c>
       <c r="G10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H10" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="I10" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="11">
@@ -1036,25 +1000,28 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D11" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" t="s">
-        <v>57</v>
-      </c>
-      <c r="F11">
-        <v>2900</v>
+        <v>58</v>
+      </c>
+      <c r="E11">
+        <v>12500</v>
+      </c>
+      <c r="F11" t="s">
+        <v>12</v>
       </c>
       <c r="G11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H11" t="s">
-        <v>58</v>
+        <v>59</v>
+      </c>
+      <c r="I11" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="12">
@@ -1062,25 +1029,28 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>61</v>
-      </c>
-      <c r="E12" t="s">
-        <v>62</v>
-      </c>
-      <c r="F12">
-        <v>3000</v>
+        <v>63</v>
+      </c>
+      <c r="E12">
+        <v>37000</v>
+      </c>
+      <c r="F12" t="s">
+        <v>12</v>
       </c>
       <c r="G12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H12" t="s">
-        <v>63</v>
+        <v>64</v>
+      </c>
+      <c r="I12" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="13">
@@ -1088,25 +1058,28 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D13" t="s">
-        <v>66</v>
-      </c>
-      <c r="E13" t="s">
-        <v>67</v>
-      </c>
-      <c r="F13">
-        <v>3100</v>
+        <v>68</v>
+      </c>
+      <c r="E13">
+        <v>29000</v>
+      </c>
+      <c r="F13" t="s">
+        <v>12</v>
       </c>
       <c r="G13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H13" t="s">
-        <v>68</v>
+        <v>69</v>
+      </c>
+      <c r="I13" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="14">
@@ -1114,25 +1087,28 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C14" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E14" t="s">
-        <v>72</v>
-      </c>
-      <c r="F14">
-        <v>3500</v>
+        <v>73</v>
+      </c>
+      <c r="E14">
+        <v>75000</v>
+      </c>
+      <c r="F14" t="s">
+        <v>24</v>
       </c>
       <c r="G14" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="H14" t="s">
-        <v>73</v>
+        <v>74</v>
+      </c>
+      <c r="I14" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="15">
@@ -1140,25 +1116,28 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D15" t="s">
-        <v>76</v>
-      </c>
-      <c r="E15" t="s">
-        <v>77</v>
-      </c>
-      <c r="F15">
-        <v>3400</v>
+        <v>78</v>
+      </c>
+      <c r="E15">
+        <v>48000</v>
+      </c>
+      <c r="F15" t="s">
+        <v>12</v>
       </c>
       <c r="G15" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H15" t="s">
-        <v>78</v>
+        <v>79</v>
+      </c>
+      <c r="I15" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="16">
@@ -1166,25 +1145,28 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D16" t="s">
-        <v>81</v>
-      </c>
-      <c r="E16" t="s">
-        <v>82</v>
-      </c>
-      <c r="F16">
-        <v>3000</v>
+        <v>83</v>
+      </c>
+      <c r="E16">
+        <v>26000</v>
+      </c>
+      <c r="F16" t="s">
+        <v>12</v>
       </c>
       <c r="G16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H16" t="s">
-        <v>83</v>
+        <v>19</v>
+      </c>
+      <c r="I16" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="17">
@@ -1192,25 +1174,28 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D17" t="s">
-        <v>86</v>
-      </c>
-      <c r="E17" t="s">
         <v>87</v>
       </c>
-      <c r="F17">
-        <v>3300</v>
+      <c r="E17">
+        <v>33000</v>
+      </c>
+      <c r="F17" t="s">
+        <v>12</v>
       </c>
       <c r="G17" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H17" t="s">
         <v>88</v>
+      </c>
+      <c r="I17" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="18">
@@ -1218,24 +1203,27 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D18" t="s">
-        <v>91</v>
-      </c>
-      <c r="E18" t="s">
         <v>92</v>
       </c>
-      <c r="F18">
-        <v>3200</v>
+      <c r="E18">
+        <v>19500</v>
+      </c>
+      <c r="F18" t="s">
+        <v>12</v>
       </c>
       <c r="G18" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H18" t="s">
+        <v>34</v>
+      </c>
+      <c r="I18" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1252,16 +1240,19 @@
       <c r="D19" t="s">
         <v>96</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19">
+        <v>85000</v>
+      </c>
+      <c r="F19" t="s">
+        <v>24</v>
+      </c>
+      <c r="G19" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" t="s">
         <v>97</v>
       </c>
-      <c r="F19">
-        <v>3600</v>
-      </c>
-      <c r="G19" t="s">
-        <v>23</v>
-      </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1278,16 +1269,19 @@
       <c r="D20" t="s">
         <v>101</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20">
+        <v>65000</v>
+      </c>
+      <c r="F20" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" t="s">
         <v>102</v>
       </c>
-      <c r="F20">
-        <v>4000</v>
-      </c>
-      <c r="G20" t="s">
-        <v>12</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1302,19 +1296,22 @@
         <v>105</v>
       </c>
       <c r="D21" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21">
+        <v>21000</v>
+      </c>
+      <c r="F21" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" t="s">
+        <v>49</v>
+      </c>
+      <c r="I21" t="s">
         <v>106</v>
-      </c>
-      <c r="E21" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21">
-        <v>2900</v>
-      </c>
-      <c r="G21" t="s">
-        <v>12</v>
-      </c>
-      <c r="H21" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="22">
@@ -1322,25 +1319,28 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
+        <v>107</v>
+      </c>
+      <c r="C22" t="s">
         <v>108</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>109</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22">
+        <v>58000</v>
+      </c>
+      <c r="F22" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" t="s">
         <v>110</v>
       </c>
-      <c r="E22" t="s">
+      <c r="I22" t="s">
         <v>111</v>
-      </c>
-      <c r="F22">
-        <v>3800</v>
-      </c>
-      <c r="G22" t="s">
-        <v>12</v>
-      </c>
-      <c r="H22" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="23">
@@ -1348,25 +1348,28 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" t="s">
         <v>113</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>114</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23">
+        <v>36000</v>
+      </c>
+      <c r="F23" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" t="s">
         <v>115</v>
       </c>
-      <c r="E23" t="s">
+      <c r="I23" t="s">
         <v>116</v>
-      </c>
-      <c r="F23">
-        <v>3500</v>
-      </c>
-      <c r="G23" t="s">
-        <v>12</v>
-      </c>
-      <c r="H23" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="24">
@@ -1374,25 +1377,28 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
+        <v>117</v>
+      </c>
+      <c r="C24" t="s">
         <v>118</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>119</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24">
+        <v>40000</v>
+      </c>
+      <c r="F24" t="s">
+        <v>24</v>
+      </c>
+      <c r="G24" t="s">
+        <v>13</v>
+      </c>
+      <c r="H24" t="s">
+        <v>25</v>
+      </c>
+      <c r="I24" t="s">
         <v>120</v>
-      </c>
-      <c r="E24" t="s">
-        <v>121</v>
-      </c>
-      <c r="F24">
-        <v>3700</v>
-      </c>
-      <c r="G24" t="s">
-        <v>23</v>
-      </c>
-      <c r="H24" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="25">
@@ -1400,25 +1406,28 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" t="s">
+        <v>122</v>
+      </c>
+      <c r="D25" t="s">
         <v>123</v>
       </c>
-      <c r="C25" t="s">
+      <c r="E25">
+        <v>32000</v>
+      </c>
+      <c r="F25" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" t="s">
         <v>124</v>
       </c>
-      <c r="D25" t="s">
+      <c r="I25" t="s">
         <v>125</v>
-      </c>
-      <c r="E25" t="s">
-        <v>126</v>
-      </c>
-      <c r="F25">
-        <v>3600</v>
-      </c>
-      <c r="G25" t="s">
-        <v>12</v>
-      </c>
-      <c r="H25" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="26">
@@ -1426,25 +1435,28 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
+        <v>126</v>
+      </c>
+      <c r="C26" t="s">
+        <v>127</v>
+      </c>
+      <c r="D26" t="s">
         <v>128</v>
       </c>
-      <c r="C26" t="s">
+      <c r="E26">
+        <v>44000</v>
+      </c>
+      <c r="F26" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" t="s">
         <v>129</v>
       </c>
-      <c r="D26" t="s">
+      <c r="I26" t="s">
         <v>130</v>
-      </c>
-      <c r="E26" t="s">
-        <v>131</v>
-      </c>
-      <c r="F26">
-        <v>3500</v>
-      </c>
-      <c r="G26" t="s">
-        <v>12</v>
-      </c>
-      <c r="H26" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="27">
@@ -1452,25 +1464,28 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
+        <v>131</v>
+      </c>
+      <c r="C27" t="s">
+        <v>132</v>
+      </c>
+      <c r="D27" t="s">
         <v>133</v>
       </c>
-      <c r="C27" t="s">
+      <c r="E27">
+        <v>17500</v>
+      </c>
+      <c r="F27" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27" t="s">
+        <v>59</v>
+      </c>
+      <c r="I27" t="s">
         <v>134</v>
-      </c>
-      <c r="D27" t="s">
-        <v>135</v>
-      </c>
-      <c r="E27" t="s">
-        <v>136</v>
-      </c>
-      <c r="F27">
-        <v>3300</v>
-      </c>
-      <c r="G27" t="s">
-        <v>12</v>
-      </c>
-      <c r="H27" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="28">
@@ -1478,25 +1493,28 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
+        <v>135</v>
+      </c>
+      <c r="C28" t="s">
+        <v>136</v>
+      </c>
+      <c r="D28" t="s">
+        <v>137</v>
+      </c>
+      <c r="E28">
+        <v>72000</v>
+      </c>
+      <c r="F28" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H28" t="s">
         <v>138</v>
       </c>
-      <c r="C28" t="s">
+      <c r="I28" t="s">
         <v>139</v>
-      </c>
-      <c r="D28" t="s">
-        <v>140</v>
-      </c>
-      <c r="E28" t="s">
-        <v>141</v>
-      </c>
-      <c r="F28">
-        <v>4200</v>
-      </c>
-      <c r="G28" t="s">
-        <v>12</v>
-      </c>
-      <c r="H28" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="29">
@@ -1504,25 +1522,28 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
+        <v>140</v>
+      </c>
+      <c r="C29" t="s">
+        <v>141</v>
+      </c>
+      <c r="D29" t="s">
+        <v>142</v>
+      </c>
+      <c r="E29">
+        <v>23000</v>
+      </c>
+      <c r="F29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" t="s">
+        <v>13</v>
+      </c>
+      <c r="H29" t="s">
+        <v>44</v>
+      </c>
+      <c r="I29" t="s">
         <v>143</v>
-      </c>
-      <c r="C29" t="s">
-        <v>144</v>
-      </c>
-      <c r="D29" t="s">
-        <v>145</v>
-      </c>
-      <c r="E29" t="s">
-        <v>146</v>
-      </c>
-      <c r="F29">
-        <v>2800</v>
-      </c>
-      <c r="G29" t="s">
-        <v>12</v>
-      </c>
-      <c r="H29" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="30">
@@ -1530,25 +1551,28 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C30" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D30" t="s">
-        <v>150</v>
-      </c>
-      <c r="E30" t="s">
         <v>11</v>
       </c>
-      <c r="F30">
-        <v>3000</v>
+      <c r="E30">
+        <v>92000</v>
+      </c>
+      <c r="F30" t="s">
+        <v>24</v>
       </c>
       <c r="G30" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="H30" t="s">
-        <v>151</v>
+        <v>146</v>
+      </c>
+      <c r="I30" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="31">
@@ -1556,25 +1580,28 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
+        <v>148</v>
+      </c>
+      <c r="C31" t="s">
+        <v>149</v>
+      </c>
+      <c r="D31" t="s">
+        <v>150</v>
+      </c>
+      <c r="E31">
+        <v>39000</v>
+      </c>
+      <c r="F31" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" t="s">
+        <v>151</v>
+      </c>
+      <c r="I31" t="s">
         <v>152</v>
-      </c>
-      <c r="C31" t="s">
-        <v>153</v>
-      </c>
-      <c r="D31" t="s">
-        <v>154</v>
-      </c>
-      <c r="E31" t="s">
-        <v>155</v>
-      </c>
-      <c r="F31">
-        <v>3400</v>
-      </c>
-      <c r="G31" t="s">
-        <v>12</v>
-      </c>
-      <c r="H31" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="32">
@@ -1582,25 +1609,28 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C32" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D32" t="s">
-        <v>159</v>
-      </c>
-      <c r="E32" t="s">
-        <v>160</v>
-      </c>
-      <c r="F32">
-        <v>3100</v>
+        <v>155</v>
+      </c>
+      <c r="E32">
+        <v>27000</v>
+      </c>
+      <c r="F32" t="s">
+        <v>12</v>
       </c>
       <c r="G32" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H32" t="s">
-        <v>161</v>
+        <v>49</v>
+      </c>
+      <c r="I32" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="33">
@@ -1608,25 +1638,28 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="C33" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="D33" t="s">
-        <v>164</v>
-      </c>
-      <c r="E33" t="s">
-        <v>165</v>
-      </c>
-      <c r="F33">
-        <v>3900</v>
+        <v>159</v>
+      </c>
+      <c r="E33">
+        <v>55000</v>
+      </c>
+      <c r="F33" t="s">
+        <v>12</v>
       </c>
       <c r="G33" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H33" t="s">
-        <v>166</v>
+        <v>160</v>
+      </c>
+      <c r="I33" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="34">
@@ -1634,25 +1667,28 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="C34" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="D34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E34" t="s">
-        <v>116</v>
-      </c>
-      <c r="F34">
-        <v>3500</v>
+        <v>114</v>
+      </c>
+      <c r="E34">
+        <v>31000</v>
+      </c>
+      <c r="F34" t="s">
+        <v>12</v>
       </c>
       <c r="G34" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H34" t="s">
-        <v>170</v>
+        <v>69</v>
+      </c>
+      <c r="I34" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="35">
@@ -1660,25 +1696,28 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C35" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D35" t="s">
-        <v>173</v>
-      </c>
-      <c r="E35" t="s">
-        <v>174</v>
-      </c>
-      <c r="F35">
-        <v>3300</v>
+        <v>167</v>
+      </c>
+      <c r="E35">
+        <v>43000</v>
+      </c>
+      <c r="F35" t="s">
+        <v>12</v>
       </c>
       <c r="G35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H35" t="s">
-        <v>175</v>
+        <v>14</v>
+      </c>
+      <c r="I35" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="36">
@@ -1686,25 +1725,28 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="C36" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="D36" t="s">
-        <v>178</v>
-      </c>
-      <c r="E36" t="s">
-        <v>179</v>
-      </c>
-      <c r="F36">
-        <v>3600</v>
+        <v>171</v>
+      </c>
+      <c r="E36">
+        <v>60000</v>
+      </c>
+      <c r="F36" t="s">
+        <v>24</v>
       </c>
       <c r="G36" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="H36" t="s">
-        <v>180</v>
+        <v>59</v>
+      </c>
+      <c r="I36" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="37">
@@ -1712,25 +1754,28 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C37" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="D37" t="s">
-        <v>183</v>
-      </c>
-      <c r="E37" t="s">
-        <v>72</v>
-      </c>
-      <c r="F37">
-        <v>3500</v>
+        <v>73</v>
+      </c>
+      <c r="E37">
+        <v>38000</v>
+      </c>
+      <c r="F37" t="s">
+        <v>12</v>
       </c>
       <c r="G37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H37" t="s">
-        <v>184</v>
+        <v>39</v>
+      </c>
+      <c r="I37" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="38">
@@ -1738,25 +1783,28 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="C38" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="D38" t="s">
-        <v>187</v>
-      </c>
-      <c r="E38" t="s">
-        <v>188</v>
-      </c>
-      <c r="F38">
-        <v>3400</v>
+        <v>178</v>
+      </c>
+      <c r="E38">
+        <v>29500</v>
+      </c>
+      <c r="F38" t="s">
+        <v>12</v>
       </c>
       <c r="G38" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H38" t="s">
-        <v>189</v>
+        <v>19</v>
+      </c>
+      <c r="I38" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="39">
@@ -1764,25 +1812,28 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="C39" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D39" t="s">
-        <v>192</v>
-      </c>
-      <c r="E39" t="s">
-        <v>193</v>
-      </c>
-      <c r="F39">
-        <v>3600</v>
+        <v>182</v>
+      </c>
+      <c r="E39">
+        <v>46000</v>
+      </c>
+      <c r="F39" t="s">
+        <v>12</v>
       </c>
       <c r="G39" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H39" t="s">
-        <v>194</v>
+        <v>64</v>
+      </c>
+      <c r="I39" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="40">
@@ -1790,25 +1841,28 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="C40" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D40" t="s">
-        <v>197</v>
-      </c>
-      <c r="E40" t="s">
-        <v>198</v>
-      </c>
-      <c r="F40">
-        <v>3500</v>
+        <v>186</v>
+      </c>
+      <c r="E40">
+        <v>51000</v>
+      </c>
+      <c r="F40" t="s">
+        <v>12</v>
       </c>
       <c r="G40" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H40" t="s">
-        <v>199</v>
+        <v>79</v>
+      </c>
+      <c r="I40" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="41">
@@ -1816,25 +1870,28 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="C41" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="D41" t="s">
-        <v>202</v>
-      </c>
-      <c r="E41" t="s">
-        <v>203</v>
-      </c>
-      <c r="F41">
-        <v>4000</v>
+        <v>190</v>
+      </c>
+      <c r="E41">
+        <v>68000</v>
+      </c>
+      <c r="F41" t="s">
+        <v>12</v>
       </c>
       <c r="G41" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H41" t="s">
-        <v>204</v>
+        <v>30</v>
+      </c>
+      <c r="I41" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="42">
@@ -1842,25 +1899,28 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>205</v>
+        <v>192</v>
       </c>
       <c r="C42" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="D42" t="s">
-        <v>207</v>
-      </c>
-      <c r="E42" t="s">
-        <v>208</v>
-      </c>
-      <c r="F42">
-        <v>2900</v>
+        <v>194</v>
+      </c>
+      <c r="E42">
+        <v>48000</v>
+      </c>
+      <c r="F42" t="s">
+        <v>24</v>
       </c>
       <c r="G42" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="H42" t="s">
-        <v>209</v>
+        <v>34</v>
+      </c>
+      <c r="I42" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="43">
@@ -1868,25 +1928,28 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="C43" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="D43" t="s">
-        <v>212</v>
-      </c>
-      <c r="E43" t="s">
-        <v>188</v>
-      </c>
-      <c r="F43">
-        <v>3300</v>
+        <v>178</v>
+      </c>
+      <c r="E43">
+        <v>24000</v>
+      </c>
+      <c r="F43" t="s">
+        <v>12</v>
       </c>
       <c r="G43" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H43" t="s">
-        <v>213</v>
+        <v>25</v>
+      </c>
+      <c r="I43" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="44">
@@ -1894,25 +1957,28 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="C44" t="s">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="D44" t="s">
-        <v>216</v>
-      </c>
-      <c r="E44" t="s">
-        <v>217</v>
-      </c>
-      <c r="F44">
-        <v>3400</v>
+        <v>201</v>
+      </c>
+      <c r="E44">
+        <v>35500</v>
+      </c>
+      <c r="F44" t="s">
+        <v>12</v>
       </c>
       <c r="G44" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H44" t="s">
-        <v>218</v>
+        <v>88</v>
+      </c>
+      <c r="I44" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="45">
@@ -1920,25 +1986,28 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>219</v>
+        <v>203</v>
       </c>
       <c r="C45" t="s">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="D45" t="s">
-        <v>221</v>
-      </c>
-      <c r="E45" t="s">
-        <v>222</v>
-      </c>
-      <c r="F45">
-        <v>3200</v>
+        <v>205</v>
+      </c>
+      <c r="E45">
+        <v>31500</v>
+      </c>
+      <c r="F45" t="s">
+        <v>12</v>
       </c>
       <c r="G45" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H45" t="s">
-        <v>223</v>
+        <v>129</v>
+      </c>
+      <c r="I45" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="46">
@@ -1946,25 +2015,28 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>224</v>
+        <v>207</v>
       </c>
       <c r="C46" t="s">
-        <v>225</v>
+        <v>208</v>
       </c>
       <c r="D46" t="s">
-        <v>226</v>
-      </c>
-      <c r="E46" t="s">
-        <v>227</v>
-      </c>
-      <c r="F46">
-        <v>3000</v>
+        <v>209</v>
+      </c>
+      <c r="E46">
+        <v>22500</v>
+      </c>
+      <c r="F46" t="s">
+        <v>12</v>
       </c>
       <c r="G46" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H46" t="s">
-        <v>228</v>
+        <v>49</v>
+      </c>
+      <c r="I46" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="47">
@@ -1972,25 +2044,28 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="C47" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="D47" t="s">
-        <v>231</v>
-      </c>
-      <c r="E47" t="s">
-        <v>232</v>
-      </c>
-      <c r="F47">
-        <v>3700</v>
+        <v>213</v>
+      </c>
+      <c r="E47">
+        <v>65000</v>
+      </c>
+      <c r="F47" t="s">
+        <v>24</v>
       </c>
       <c r="G47" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="H47" t="s">
-        <v>233</v>
+        <v>74</v>
+      </c>
+      <c r="I47" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="48">
@@ -1998,25 +2073,28 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>234</v>
+        <v>215</v>
       </c>
       <c r="C48" t="s">
-        <v>235</v>
+        <v>216</v>
       </c>
       <c r="D48" t="s">
-        <v>236</v>
-      </c>
-      <c r="E48" t="s">
-        <v>237</v>
-      </c>
-      <c r="F48">
-        <v>2900</v>
+        <v>217</v>
+      </c>
+      <c r="E48">
+        <v>18500</v>
+      </c>
+      <c r="F48" t="s">
+        <v>12</v>
       </c>
       <c r="G48" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H48" t="s">
-        <v>238</v>
+        <v>34</v>
+      </c>
+      <c r="I48" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="49">
@@ -2024,25 +2102,28 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="C49" t="s">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="D49" t="s">
-        <v>241</v>
-      </c>
-      <c r="E49" t="s">
-        <v>242</v>
-      </c>
-      <c r="F49">
-        <v>3500</v>
+        <v>221</v>
+      </c>
+      <c r="E49">
+        <v>47000</v>
+      </c>
+      <c r="F49" t="s">
+        <v>12</v>
       </c>
       <c r="G49" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H49" t="s">
-        <v>243</v>
+        <v>124</v>
+      </c>
+      <c r="I49" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="50">
@@ -2050,25 +2131,28 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>244</v>
+        <v>223</v>
       </c>
       <c r="C50" t="s">
-        <v>245</v>
+        <v>224</v>
       </c>
       <c r="D50" t="s">
-        <v>246</v>
-      </c>
-      <c r="E50" t="s">
-        <v>126</v>
-      </c>
-      <c r="F50">
-        <v>3600</v>
+        <v>123</v>
+      </c>
+      <c r="E50">
+        <v>38500</v>
+      </c>
+      <c r="F50" t="s">
+        <v>12</v>
       </c>
       <c r="G50" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H50" t="s">
-        <v>247</v>
+        <v>102</v>
+      </c>
+      <c r="I50" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="51">
@@ -2076,25 +2160,28 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>248</v>
+        <v>226</v>
       </c>
       <c r="C51" t="s">
-        <v>249</v>
+        <v>227</v>
       </c>
       <c r="D51" t="s">
-        <v>250</v>
-      </c>
-      <c r="E51" t="s">
-        <v>251</v>
-      </c>
-      <c r="F51">
-        <v>3500</v>
+        <v>228</v>
+      </c>
+      <c r="E51">
+        <v>42000</v>
+      </c>
+      <c r="F51" t="s">
+        <v>12</v>
       </c>
       <c r="G51" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H51" t="s">
-        <v>29</v>
+        <v>44</v>
+      </c>
+      <c r="I51" t="s">
+        <v>229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>